<commit_message>
Day 09: Date and Time Formulas
</commit_message>
<xml_diff>
--- a/Excel/Day 08/Excel-Practice-(Day-08).xlsx
+++ b/Excel/Day 08/Excel-Practice-(Day-08).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Analyst\Excel\Day 08\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FAFCC7C9-3447-4460-B9DE-EE50D6DD5F6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C59B76EB-226E-4E1E-A624-C0FE495F42D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="678" firstSheet="14" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="678" firstSheet="15" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw Data" sheetId="1" r:id="rId1"/>
@@ -23,12 +23,15 @@
     <sheet name="fill" sheetId="9" r:id="rId8"/>
     <sheet name="Go to Special" sheetId="10" r:id="rId9"/>
     <sheet name="Paste Special With Find&amp;Replace" sheetId="11" r:id="rId10"/>
-    <sheet name="Clear" sheetId="12" r:id="rId11"/>
-    <sheet name="Cell Referencing" sheetId="13" r:id="rId12"/>
-    <sheet name="Text Formulas Notes" sheetId="14" r:id="rId13"/>
-    <sheet name="Text Formulas Practice" sheetId="15" r:id="rId14"/>
-    <sheet name="Statistical Formulas Notes" sheetId="16" r:id="rId15"/>
-    <sheet name="Statistical Formulas Practice" sheetId="17" r:id="rId16"/>
+    <sheet name="Sheet1" sheetId="18" r:id="rId11"/>
+    <sheet name="Clear" sheetId="12" r:id="rId12"/>
+    <sheet name="Cell Referencing" sheetId="13" r:id="rId13"/>
+    <sheet name="Text Formulas Notes" sheetId="14" r:id="rId14"/>
+    <sheet name="Text Formulas Practice" sheetId="15" r:id="rId15"/>
+    <sheet name="Statistical Formulas Notes" sheetId="16" r:id="rId16"/>
+    <sheet name="Sheet2" sheetId="19" r:id="rId17"/>
+    <sheet name="Statistical Formulas Practice" sheetId="17" r:id="rId18"/>
+    <sheet name=" Formulas Notes" sheetId="20" r:id="rId19"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Filter!$A$1:$F$38</definedName>
@@ -42,8 +45,8 @@
     </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{46BE6895-7355-4a93-B00E-2C351335B9C9}">
       <x15:slicerCaches xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main">
-        <x14:slicerCache r:id="rId17"/>
-        <x14:slicerCache r:id="rId18"/>
+        <x14:slicerCache r:id="rId20"/>
+        <x14:slicerCache r:id="rId21"/>
       </x15:slicerCaches>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -85,7 +88,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4385" uniqueCount="907">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4403" uniqueCount="915">
   <si>
     <t>Employee_ID</t>
   </si>
@@ -2807,6 +2810,30 @@
   </si>
   <si>
     <t>INTEGER,TRUNC</t>
+  </si>
+  <si>
+    <t>CEILING</t>
+  </si>
+  <si>
+    <t>CEILING(number, significance)</t>
+  </si>
+  <si>
+    <t>Number ko next specified multiple tak round up karta hai</t>
+  </si>
+  <si>
+    <t>Price/quantity rounding</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =CEILING(12.3,1) → 13</t>
+  </si>
+  <si>
+    <t>FLOOR,CEILING,MROUND</t>
+  </si>
+  <si>
+    <t>ABS, MOD, POWER, SQRT</t>
+  </si>
+  <si>
+    <t>-ABS</t>
   </si>
 </sst>
 </file>
@@ -2820,7 +2847,7 @@
     <numFmt numFmtId="167" formatCode="&quot;Rs. &quot;#,##0"/>
     <numFmt numFmtId="168" formatCode="&quot;Rs.&quot;\ #,##0"/>
   </numFmts>
-  <fonts count="30" x14ac:knownFonts="1">
+  <fonts count="31" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3036,6 +3063,13 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="35">
@@ -4111,7 +4145,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="265">
+  <cellXfs count="268">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4825,6 +4859,15 @@
     <xf numFmtId="0" fontId="22" fillId="27" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="27" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4848,6 +4891,152 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="2"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="4" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="2"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="2"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5653,152 +5842,6 @@
         <top/>
         <bottom/>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="2"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="4" tint="-0.24994659260841701"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="2"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="2"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -6732,15 +6775,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2688C5AF-1E0A-4EDD-AF11-5A4BBABB9721}" name="Employees" displayName="Employees" ref="A1:F39" totalsRowCount="1" headerRowDxfId="45" dataDxfId="43" headerRowBorderDxfId="44" tableBorderDxfId="42">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2688C5AF-1E0A-4EDD-AF11-5A4BBABB9721}" name="Employees" displayName="Employees" ref="A1:F39" totalsRowCount="1" headerRowDxfId="59" dataDxfId="57" headerRowBorderDxfId="58" tableBorderDxfId="56">
   <autoFilter ref="A1:F38" xr:uid="{2688C5AF-1E0A-4EDD-AF11-5A4BBABB9721}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B1033A5F-C26D-48E8-B4BE-5F7761A770FB}" name="Date" dataDxfId="41" totalsRowDxfId="40"/>
-    <tableColumn id="2" xr3:uid="{AD6BA12D-25CE-4D3E-8E2A-1DD281A3FDA5}" name="Employee Name" dataDxfId="39" totalsRowDxfId="38"/>
-    <tableColumn id="3" xr3:uid="{96E1CF2B-482C-42D2-8CEA-C0CE6D69979C}" name="Department" dataDxfId="37" totalsRowDxfId="36"/>
-    <tableColumn id="4" xr3:uid="{602E6D48-4D10-4D1E-9636-6A41FF0A4753}" name="Region" dataDxfId="35" totalsRowDxfId="34"/>
-    <tableColumn id="5" xr3:uid="{98D904BD-DEE8-4674-A97B-995E27B5AB23}" name="Sales (Rs.)" dataDxfId="33" totalsRowDxfId="32"/>
-    <tableColumn id="6" xr3:uid="{F7A5EC06-42D8-4DD0-83BA-C91339988D38}" name="Target (Rs.)" totalsRowFunction="custom" dataDxfId="31" totalsRowDxfId="30">
+    <tableColumn id="1" xr3:uid="{B1033A5F-C26D-48E8-B4BE-5F7761A770FB}" name="Date" dataDxfId="55" totalsRowDxfId="54"/>
+    <tableColumn id="2" xr3:uid="{AD6BA12D-25CE-4D3E-8E2A-1DD281A3FDA5}" name="Employee Name" dataDxfId="53" totalsRowDxfId="52"/>
+    <tableColumn id="3" xr3:uid="{96E1CF2B-482C-42D2-8CEA-C0CE6D69979C}" name="Department" dataDxfId="51" totalsRowDxfId="50"/>
+    <tableColumn id="4" xr3:uid="{602E6D48-4D10-4D1E-9636-6A41FF0A4753}" name="Region" dataDxfId="49" totalsRowDxfId="48"/>
+    <tableColumn id="5" xr3:uid="{98D904BD-DEE8-4674-A97B-995E27B5AB23}" name="Sales (Rs.)" dataDxfId="47" totalsRowDxfId="46"/>
+    <tableColumn id="6" xr3:uid="{F7A5EC06-42D8-4DD0-83BA-C91339988D38}" name="Target (Rs.)" totalsRowFunction="custom" dataDxfId="45" totalsRowDxfId="44">
       <totalsRowFormula>SUM(F2:F38)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -7033,7 +7076,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="350" row="3">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="2">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -19535,7 +19578,7 @@
       </c>
       <c r="H3" s="135">
         <f t="shared" ref="H3:H16" ca="1" si="1">(RANDBETWEEN(10,50))/100</f>
-        <v>0.46</v>
+        <v>0.3</v>
       </c>
       <c r="I3" s="105">
         <v>100</v>
@@ -19580,7 +19623,7 @@
       </c>
       <c r="H4" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.26</v>
+        <v>0.3</v>
       </c>
       <c r="X4" s="105" t="str">
         <f t="shared" si="0"/>
@@ -19600,7 +19643,7 @@
       </c>
       <c r="AB4" s="135">
         <f t="shared" ca="1" si="2"/>
-        <v>0.46</v>
+        <v>0.3</v>
       </c>
       <c r="AC4" s="105">
         <f t="shared" si="2"/>
@@ -19622,7 +19665,7 @@
       </c>
       <c r="H5" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.33</v>
+        <v>0.18</v>
       </c>
       <c r="X5" s="105" t="str">
         <f t="shared" si="0"/>
@@ -19642,7 +19685,7 @@
       </c>
       <c r="AB5" s="135">
         <f t="shared" ref="AB5:AB17" ca="1" si="6">H4</f>
-        <v>0.26</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="6" spans="4:29" x14ac:dyDescent="0.25">
@@ -19660,7 +19703,7 @@
       </c>
       <c r="H6" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.46</v>
+        <v>0.25</v>
       </c>
       <c r="L6" s="246" t="s">
         <v>540</v>
@@ -19692,7 +19735,7 @@
       </c>
       <c r="AB6" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.33</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="7" spans="4:29" x14ac:dyDescent="0.25">
@@ -19710,7 +19753,7 @@
       </c>
       <c r="H7" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.11</v>
+        <v>0.26</v>
       </c>
       <c r="X7" s="105" t="str">
         <f t="shared" si="0"/>
@@ -19730,7 +19773,7 @@
       </c>
       <c r="AB7" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.46</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="8" spans="4:29" x14ac:dyDescent="0.25">
@@ -19748,7 +19791,7 @@
       </c>
       <c r="H8" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.18</v>
+        <v>0.41</v>
       </c>
       <c r="M8" s="105">
         <v>137196</v>
@@ -19774,7 +19817,7 @@
       </c>
       <c r="AB8" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.11</v>
+        <v>0.26</v>
       </c>
     </row>
     <row r="9" spans="4:29" x14ac:dyDescent="0.25">
@@ -19792,7 +19835,7 @@
       </c>
       <c r="H9" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.19</v>
+        <v>0.11</v>
       </c>
       <c r="M9" s="105">
         <v>64256</v>
@@ -19816,7 +19859,7 @@
       </c>
       <c r="AB9" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.18</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="10" spans="4:29" x14ac:dyDescent="0.25">
@@ -19834,7 +19877,7 @@
       </c>
       <c r="H10" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.16</v>
+        <v>0.25</v>
       </c>
       <c r="M10" s="105">
         <v>137080</v>
@@ -19860,7 +19903,7 @@
       </c>
       <c r="AB10" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.19</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="11" spans="4:29" x14ac:dyDescent="0.25">
@@ -19878,7 +19921,7 @@
       </c>
       <c r="H11" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.21</v>
+        <v>0.36</v>
       </c>
       <c r="M11" s="105">
         <v>95302</v>
@@ -19904,7 +19947,7 @@
       </c>
       <c r="AB11" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.16</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="12" spans="4:29" x14ac:dyDescent="0.25">
@@ -19922,7 +19965,7 @@
       </c>
       <c r="H12" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.35</v>
+        <v>0.46</v>
       </c>
       <c r="M12" s="105">
         <v>68657</v>
@@ -19948,7 +19991,7 @@
       </c>
       <c r="AB12" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.21</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="13" spans="4:29" x14ac:dyDescent="0.25">
@@ -19966,7 +20009,7 @@
       </c>
       <c r="H13" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.46</v>
+        <v>0.31</v>
       </c>
       <c r="M13" s="105">
         <v>66062</v>
@@ -19992,7 +20035,7 @@
       </c>
       <c r="AB13" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.35</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="14" spans="4:29" x14ac:dyDescent="0.25">
@@ -20010,7 +20053,7 @@
       </c>
       <c r="H14" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.23</v>
+        <v>0.28999999999999998</v>
       </c>
       <c r="M14" s="105">
         <v>98878</v>
@@ -20036,7 +20079,7 @@
       </c>
       <c r="AB14" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.46</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="15" spans="4:29" x14ac:dyDescent="0.25">
@@ -20054,7 +20097,7 @@
       </c>
       <c r="H15" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.12</v>
+        <v>0.31</v>
       </c>
       <c r="M15" s="105">
         <v>40851</v>
@@ -20080,7 +20123,7 @@
       </c>
       <c r="AB15" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.23</v>
+        <v>0.28999999999999998</v>
       </c>
     </row>
     <row r="16" spans="4:29" x14ac:dyDescent="0.25">
@@ -20098,7 +20141,7 @@
       </c>
       <c r="H16" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.4</v>
+        <v>0.34</v>
       </c>
       <c r="M16" s="105"/>
       <c r="N16" s="105"/>
@@ -20120,7 +20163,7 @@
       </c>
       <c r="AB16" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.12</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="17" spans="4:28" x14ac:dyDescent="0.25">
@@ -20149,7 +20192,7 @@
       </c>
       <c r="AB17" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.4</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="18" spans="4:28" x14ac:dyDescent="0.25">
@@ -20731,6 +20774,15 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8143E889-3392-483F-BF6D-D6C07987CB32}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{404D2EFD-B6FA-4B0F-ADC3-3722B7ACA4BB}">
   <dimension ref="A4:AB56"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -23243,7 +23295,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{434A35C9-1881-44D8-8A07-81190F12B4B5}">
   <dimension ref="B3:M41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -24442,7 +24494,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C639D35D-42B3-4FB6-B1C2-2E99B2FC7CC6}">
   <dimension ref="B2:G24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -24894,7 +24946,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BD5D473-BB1A-4083-B1E9-1F028EFD68A4}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
@@ -26940,15 +26992,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B54A3611-4A04-4C13-950D-B1A57B926186}">
-  <dimension ref="B3:G33"/>
+  <dimension ref="B3:G34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" customWidth="1"/>
     <col min="2" max="2" width="8.5703125" customWidth="1"/>
     <col min="3" max="3" width="18.140625" customWidth="1"/>
-    <col min="4" max="5" width="36.140625" customWidth="1"/>
+    <col min="4" max="4" width="36.140625" customWidth="1"/>
+    <col min="5" max="5" width="52.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="28.5703125" customWidth="1"/>
     <col min="7" max="7" width="41.85546875" customWidth="1"/>
   </cols>
@@ -27554,31 +27607,60 @@
       </c>
     </row>
     <row r="33" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B33" s="261" t="s">
+      <c r="B33" s="214">
+        <v>30</v>
+      </c>
+      <c r="C33" s="215" t="s">
+        <v>907</v>
+      </c>
+      <c r="D33" s="212" t="s">
+        <v>908</v>
+      </c>
+      <c r="E33" s="212" t="s">
+        <v>909</v>
+      </c>
+      <c r="F33" s="212" t="s">
+        <v>910</v>
+      </c>
+      <c r="G33" s="213" t="s">
+        <v>911</v>
+      </c>
+    </row>
+    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B34" s="261" t="s">
         <v>898</v>
       </c>
-      <c r="C33" s="262"/>
-      <c r="D33" s="262"/>
-      <c r="E33" s="262"/>
-      <c r="F33" s="262"/>
-      <c r="G33" s="263"/>
+      <c r="C34" s="262"/>
+      <c r="D34" s="262"/>
+      <c r="E34" s="262"/>
+      <c r="F34" s="262"/>
+      <c r="G34" s="263"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B33:G33"/>
+    <mergeCell ref="B34:G34"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF7BFF78-547F-4715-AFEA-94C43A5A01BF}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98DC9442-C99E-46AE-BA24-6CDCF6B108E6}">
-  <dimension ref="A1:N54"/>
+  <dimension ref="A1:P56"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11.5703125" customWidth="1"/>
     <col min="3" max="3" width="13.140625" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" customWidth="1"/>
+    <col min="4" max="4" width="21.7109375" customWidth="1"/>
     <col min="6" max="6" width="11.5703125" customWidth="1"/>
     <col min="7" max="7" width="13.140625" customWidth="1"/>
     <col min="8" max="8" width="14.42578125" bestFit="1" customWidth="1"/>
@@ -27586,6 +27668,9 @@
     <col min="11" max="11" width="13.140625" customWidth="1"/>
     <col min="12" max="12" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="12.42578125" customWidth="1"/>
+    <col min="14" max="14" width="16.140625" customWidth="1"/>
+    <col min="15" max="15" width="13.5703125" customWidth="1"/>
+    <col min="16" max="16" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -27608,15 +27693,15 @@
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B4" s="209">
         <f t="shared" ref="B4:D13" ca="1" si="0">RAND()</f>
-        <v>0.16072348080125931</v>
+        <v>0.98102162000715853</v>
       </c>
       <c r="C4" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.75384475150803354</v>
+        <v>0.17007252180839505</v>
       </c>
       <c r="D4" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.36870332964025232</v>
+        <v>0.57474744820829327</v>
       </c>
       <c r="F4" s="167" t="s">
         <v>901</v>
@@ -27631,15 +27716,15 @@
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B5" s="209">
         <f t="shared" ca="1" si="0"/>
-        <v>0.13476323169696747</v>
+        <v>9.6311909677898599E-3</v>
       </c>
       <c r="C5" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.52370077394828962</v>
+        <v>0.81955824938253519</v>
       </c>
       <c r="D5" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.65679199020861345</v>
+        <v>0.53407946938173823</v>
       </c>
       <c r="F5" s="169">
         <v>1</v>
@@ -27655,15 +27740,15 @@
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B6" s="209">
         <f t="shared" ca="1" si="0"/>
-        <v>0.8778653970739787</v>
+        <v>0.67918303862669183</v>
       </c>
       <c r="C6" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.95180327718179625</v>
+        <v>0.48345919106540314</v>
       </c>
       <c r="D6" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.66239914437781122</v>
+        <v>0.79596393584054148</v>
       </c>
       <c r="F6" s="169">
         <v>2</v>
@@ -27679,15 +27764,15 @@
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B7" s="209">
         <f t="shared" ca="1" si="0"/>
-        <v>0.31596278131754751</v>
+        <v>0.77088336944116687</v>
       </c>
       <c r="C7" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.41184179716271396</v>
+        <v>0.53395016796660477</v>
       </c>
       <c r="D7" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.63112812865155266</v>
+        <v>0.3808545110264232</v>
       </c>
       <c r="F7" s="169">
         <v>3</v>
@@ -27703,15 +27788,15 @@
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B8" s="209">
         <f t="shared" ca="1" si="0"/>
-        <v>0.50802196321477022</v>
+        <v>0.20916300701892121</v>
       </c>
       <c r="C8" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.90168968882796763</v>
+        <v>0.33033881540727084</v>
       </c>
       <c r="D8" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.46358484573139747</v>
+        <v>0.71278704039809271</v>
       </c>
       <c r="F8" s="169">
         <v>4</v>
@@ -27727,15 +27812,15 @@
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B9" s="209">
         <f t="shared" ca="1" si="0"/>
-        <v>0.94847096584345303</v>
+        <v>0.4667868695605315</v>
       </c>
       <c r="C9" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.96334856447294026</v>
+        <v>0.43912391111478211</v>
       </c>
       <c r="D9" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.1903252033243259</v>
+        <v>0.6077545335002098</v>
       </c>
       <c r="F9" s="169">
         <v>5</v>
@@ -27751,15 +27836,15 @@
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B10" s="209">
         <f t="shared" ca="1" si="0"/>
-        <v>0.8730117237329752</v>
+        <v>0.68047145390073382</v>
       </c>
       <c r="C10" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.93214034270350299</v>
+        <v>0.25660178154108704</v>
       </c>
       <c r="D10" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.28416207615293831</v>
+        <v>0.95517078375955689</v>
       </c>
       <c r="F10" s="169">
         <v>6</v>
@@ -27775,15 +27860,15 @@
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B11" s="209">
         <f t="shared" ca="1" si="0"/>
-        <v>0.43536000754022985</v>
+        <v>0.35782091914357617</v>
       </c>
       <c r="C11" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.84686831864136602</v>
+        <v>0.13250083664789813</v>
       </c>
       <c r="D11" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.61444447125136448</v>
+        <v>0.63348071089257885</v>
       </c>
       <c r="F11" s="169">
         <v>7</v>
@@ -27799,15 +27884,15 @@
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B12" s="209">
         <f t="shared" ca="1" si="0"/>
-        <v>0.48207384630522954</v>
+        <v>0.64922694129342085</v>
       </c>
       <c r="C12" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.49525882339465155</v>
+        <v>0.40391878665197645</v>
       </c>
       <c r="D12" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.92004881192326937</v>
+        <v>8.7295619137582103E-2</v>
       </c>
       <c r="F12" s="169">
         <v>8</v>
@@ -27823,15 +27908,15 @@
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B13" s="209">
         <f t="shared" ca="1" si="0"/>
-        <v>0.47683426340050916</v>
+        <v>0.24167358552776608</v>
       </c>
       <c r="C13" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.91071465055975598</v>
+        <v>0.68510726213848183</v>
       </c>
       <c r="D13" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.37455863899222386</v>
+        <v>0.22332858198087546</v>
       </c>
       <c r="F13" s="169">
         <v>9</v>
@@ -27856,8 +27941,8 @@
         <v>214.626</v>
       </c>
     </row>
-    <row r="17" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B17" s="264" t="s">
+    <row r="17" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B17" s="266" t="s">
         <v>900</v>
       </c>
       <c r="C17" s="264"/>
@@ -27874,18 +27959,18 @@
       <c r="L17" s="260"/>
       <c r="M17" s="260"/>
     </row>
-    <row r="18" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B18" s="209">
         <f ca="1">RANDBETWEEN(0,100)</f>
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="C18" s="168">
         <f t="shared" ref="B18:D27" ca="1" si="2">RANDBETWEEN(0,100)</f>
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="D18" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>9</v>
+        <v>78</v>
       </c>
       <c r="F18" s="167" t="s">
         <v>901</v>
@@ -27909,18 +27994,18 @@
         <v>848</v>
       </c>
     </row>
-    <row r="19" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B19" s="209">
         <f t="shared" ca="1" si="2"/>
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="C19" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>91</v>
+        <v>51</v>
       </c>
       <c r="D19" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="F19" s="169">
         <v>1</v>
@@ -27947,18 +28032,18 @@
         <v>186.7</v>
       </c>
     </row>
-    <row r="20" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B20" s="209">
         <f t="shared" ca="1" si="2"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C20" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="D20" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>94</v>
+        <v>31</v>
       </c>
       <c r="F20" s="169">
         <v>2</v>
@@ -27985,18 +28070,18 @@
         <v>1134.2</v>
       </c>
     </row>
-    <row r="21" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B21" s="209">
         <f t="shared" ca="1" si="2"/>
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="C21" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="D21" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="F21" s="169">
         <v>3</v>
@@ -28023,18 +28108,18 @@
         <v>1056.2</v>
       </c>
     </row>
-    <row r="22" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B22" s="209">
         <f t="shared" ca="1" si="2"/>
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="C22" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>66</v>
+        <v>87</v>
       </c>
       <c r="D22" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>46</v>
       </c>
       <c r="F22" s="169">
         <v>4</v>
@@ -28061,18 +28146,18 @@
         <v>444.9</v>
       </c>
     </row>
-    <row r="23" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B23" s="209">
         <f t="shared" ca="1" si="2"/>
-        <v>76</v>
+        <v>39</v>
       </c>
       <c r="C23" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>84</v>
+        <v>43</v>
       </c>
       <c r="D23" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>20</v>
+        <v>53</v>
       </c>
       <c r="F23" s="169">
         <v>5</v>
@@ -28099,18 +28184,18 @@
         <v>1319.4</v>
       </c>
     </row>
-    <row r="24" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B24" s="209">
         <f t="shared" ca="1" si="2"/>
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="C24" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>49</v>
+        <v>1</v>
       </c>
       <c r="D24" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F24" s="169">
         <v>6</v>
@@ -28137,18 +28222,18 @@
         <v>226.9</v>
       </c>
     </row>
-    <row r="25" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B25" s="209">
         <f t="shared" ca="1" si="2"/>
-        <v>66</v>
+        <v>88</v>
       </c>
       <c r="C25" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>97</v>
+        <v>70</v>
       </c>
       <c r="D25" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>90</v>
+        <v>8</v>
       </c>
       <c r="F25" s="169">
         <v>7</v>
@@ -28175,18 +28260,18 @@
         <v>130.1</v>
       </c>
     </row>
-    <row r="26" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B26" s="209">
         <f t="shared" ca="1" si="2"/>
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C26" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>29</v>
+        <v>68</v>
       </c>
       <c r="D26" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="F26" s="169">
         <v>8</v>
@@ -28213,18 +28298,18 @@
         <v>351.1</v>
       </c>
     </row>
-    <row r="27" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B27" s="209">
         <f t="shared" ca="1" si="2"/>
-        <v>25</v>
+        <v>74</v>
       </c>
       <c r="C27" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>22</v>
+        <v>56</v>
       </c>
       <c r="D27" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>40</v>
+        <v>71</v>
       </c>
       <c r="F27" s="169">
         <v>9</v>
@@ -28251,7 +28336,7 @@
         <v>1433</v>
       </c>
     </row>
-    <row r="28" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:14" x14ac:dyDescent="0.25">
       <c r="F28" s="169">
         <v>10</v>
       </c>
@@ -28277,7 +28362,7 @@
         <v>214.6</v>
       </c>
     </row>
-    <row r="30" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B30" s="264" t="s">
         <v>873</v>
       </c>
@@ -28289,18 +28374,18 @@
       <c r="G30" s="260"/>
       <c r="H30" s="260"/>
     </row>
-    <row r="31" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B31" s="209" cm="1">
         <f t="array" aca="1" ref="B31:D40" ca="1">_xlfn.RANDARRAY(10,3,0,100,TRUE)</f>
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="C31" s="168">
         <f ca="1"/>
-        <v>9</v>
+        <v>72</v>
       </c>
       <c r="D31" s="168">
         <f ca="1"/>
-        <v>79</v>
+        <v>27</v>
       </c>
       <c r="F31" s="167" t="s">
         <v>901</v>
@@ -28311,19 +28396,26 @@
       <c r="H31" s="167" t="s">
         <v>904</v>
       </c>
-    </row>
-    <row r="32" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="J31" s="260" t="s">
+        <v>912</v>
+      </c>
+      <c r="K31" s="260"/>
+      <c r="L31" s="260"/>
+      <c r="M31" s="260"/>
+      <c r="N31" s="260"/>
+    </row>
+    <row r="32" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B32" s="209">
         <f ca="1"/>
-        <v>65</v>
+        <v>95</v>
       </c>
       <c r="C32" s="168">
         <f ca="1"/>
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="D32" s="168">
         <f ca="1"/>
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="F32" s="169">
         <v>1</v>
@@ -28335,19 +28427,34 @@
         <f>ROUNDDOWN(G32,3)</f>
         <v>186.74600000000001</v>
       </c>
-    </row>
-    <row r="33" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="J32" s="167" t="s">
+        <v>901</v>
+      </c>
+      <c r="K32" s="167" t="s">
+        <v>902</v>
+      </c>
+      <c r="L32" s="167" t="s">
+        <v>853</v>
+      </c>
+      <c r="M32" s="167" t="s">
+        <v>907</v>
+      </c>
+      <c r="N32" s="265" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="33" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B33" s="209">
         <f ca="1"/>
-        <v>63</v>
+        <v>25</v>
       </c>
       <c r="C33" s="168">
         <f ca="1"/>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D33" s="168">
         <f ca="1"/>
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="F33" s="169">
         <v>2</v>
@@ -28359,22 +28466,37 @@
         <f t="shared" ref="H33:H41" si="6">ROUNDDOWN(G33,3)</f>
         <v>1134.203</v>
       </c>
-      <c r="N33" t="s">
-        <v>535</v>
-      </c>
-    </row>
-    <row r="34" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="J33" s="169">
+        <v>1</v>
+      </c>
+      <c r="K33" s="168">
+        <v>49</v>
+      </c>
+      <c r="L33" s="168">
+        <f>FLOOR(K33,3)</f>
+        <v>48</v>
+      </c>
+      <c r="M33" s="168">
+        <f>CEILING(K33,3)</f>
+        <v>51</v>
+      </c>
+      <c r="N33" s="168">
+        <f>MROUND(K33,3)</f>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="34" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B34" s="209">
         <f ca="1"/>
-        <v>12</v>
+        <v>77</v>
       </c>
       <c r="C34" s="168">
         <f ca="1"/>
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="D34" s="168">
         <f ca="1"/>
-        <v>14</v>
+        <v>95</v>
       </c>
       <c r="F34" s="169">
         <v>3</v>
@@ -28386,19 +28508,37 @@
         <f t="shared" si="6"/>
         <v>1056.26</v>
       </c>
-    </row>
-    <row r="35" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="J34" s="169">
+        <v>2</v>
+      </c>
+      <c r="K34" s="168">
+        <v>92</v>
+      </c>
+      <c r="L34" s="168">
+        <f t="shared" ref="L34:L42" si="7">FLOOR(K34,3)</f>
+        <v>90</v>
+      </c>
+      <c r="M34" s="168">
+        <f t="shared" ref="M34:M42" si="8">CEILING(K34,3)</f>
+        <v>93</v>
+      </c>
+      <c r="N34" s="168">
+        <f t="shared" ref="N34:N42" si="9">MROUND(K34,3)</f>
+        <v>93</v>
+      </c>
+    </row>
+    <row r="35" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B35" s="209">
         <f ca="1"/>
-        <v>70</v>
+        <v>44</v>
       </c>
       <c r="C35" s="168">
         <f ca="1"/>
-        <v>52</v>
+        <v>31</v>
       </c>
       <c r="D35" s="168">
         <f ca="1"/>
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="F35" s="169">
         <v>4</v>
@@ -28410,19 +28550,37 @@
         <f t="shared" si="6"/>
         <v>444.95499999999998</v>
       </c>
-    </row>
-    <row r="36" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="J35" s="169">
+        <v>3</v>
+      </c>
+      <c r="K35" s="168">
+        <v>49</v>
+      </c>
+      <c r="L35" s="168">
+        <f t="shared" si="7"/>
+        <v>48</v>
+      </c>
+      <c r="M35" s="168">
+        <f t="shared" si="8"/>
+        <v>51</v>
+      </c>
+      <c r="N35" s="168">
+        <f t="shared" si="9"/>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="36" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B36" s="209">
         <f ca="1"/>
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C36" s="168">
         <f ca="1"/>
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="D36" s="168">
         <f ca="1"/>
-        <v>93</v>
+        <v>3</v>
       </c>
       <c r="F36" s="169">
         <v>5</v>
@@ -28434,19 +28592,37 @@
         <f t="shared" si="6"/>
         <v>1319.4690000000001</v>
       </c>
-    </row>
-    <row r="37" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="J36" s="169">
+        <v>4</v>
+      </c>
+      <c r="K36" s="168">
+        <v>32</v>
+      </c>
+      <c r="L36" s="168">
+        <f t="shared" si="7"/>
+        <v>30</v>
+      </c>
+      <c r="M36" s="168">
+        <f t="shared" si="8"/>
+        <v>33</v>
+      </c>
+      <c r="N36" s="168">
+        <f t="shared" si="9"/>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="37" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B37" s="209">
         <f ca="1"/>
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="C37" s="168">
         <f ca="1"/>
-        <v>36</v>
+        <v>63</v>
       </c>
       <c r="D37" s="168">
         <f ca="1"/>
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="F37" s="169">
         <v>6</v>
@@ -28458,19 +28634,37 @@
         <f t="shared" si="6"/>
         <v>226.92699999999999</v>
       </c>
-    </row>
-    <row r="38" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="J37" s="169">
+        <v>5</v>
+      </c>
+      <c r="K37" s="168">
+        <v>43</v>
+      </c>
+      <c r="L37" s="168">
+        <f t="shared" si="7"/>
+        <v>42</v>
+      </c>
+      <c r="M37" s="168">
+        <f t="shared" si="8"/>
+        <v>45</v>
+      </c>
+      <c r="N37" s="168">
+        <f t="shared" si="9"/>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="38" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B38" s="209">
         <f ca="1"/>
-        <v>35</v>
+        <v>89</v>
       </c>
       <c r="C38" s="168">
         <f ca="1"/>
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="D38" s="168">
         <f ca="1"/>
-        <v>79</v>
+        <v>27</v>
       </c>
       <c r="F38" s="169">
         <v>7</v>
@@ -28482,19 +28676,37 @@
         <f t="shared" si="6"/>
         <v>130.15899999999999</v>
       </c>
-    </row>
-    <row r="39" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="J38" s="169">
+        <v>6</v>
+      </c>
+      <c r="K38" s="168">
+        <v>57</v>
+      </c>
+      <c r="L38" s="168">
+        <f t="shared" si="7"/>
+        <v>57</v>
+      </c>
+      <c r="M38" s="168">
+        <f t="shared" si="8"/>
+        <v>57</v>
+      </c>
+      <c r="N38" s="168">
+        <f t="shared" si="9"/>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="39" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B39" s="209">
         <f ca="1"/>
-        <v>64</v>
+        <v>15</v>
       </c>
       <c r="C39" s="168">
         <f ca="1"/>
-        <v>72</v>
+        <v>22</v>
       </c>
       <c r="D39" s="168">
         <f ca="1"/>
-        <v>74</v>
+        <v>37</v>
       </c>
       <c r="F39" s="169">
         <v>8</v>
@@ -28506,19 +28718,37 @@
         <f t="shared" si="6"/>
         <v>351.12700000000001</v>
       </c>
-    </row>
-    <row r="40" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="J39" s="169">
+        <v>7</v>
+      </c>
+      <c r="K39" s="168">
+        <v>45</v>
+      </c>
+      <c r="L39" s="168">
+        <f t="shared" si="7"/>
+        <v>45</v>
+      </c>
+      <c r="M39" s="168">
+        <f t="shared" si="8"/>
+        <v>45</v>
+      </c>
+      <c r="N39" s="168">
+        <f t="shared" si="9"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="40" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B40" s="209">
         <f ca="1"/>
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="C40" s="168">
         <f ca="1"/>
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="D40" s="168">
         <f ca="1"/>
-        <v>19</v>
+        <v>97</v>
       </c>
       <c r="F40" s="169">
         <v>9</v>
@@ -28530,8 +28760,26 @@
         <f t="shared" si="6"/>
         <v>1433.059</v>
       </c>
-    </row>
-    <row r="41" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="J40" s="169">
+        <v>8</v>
+      </c>
+      <c r="K40" s="168">
+        <v>59</v>
+      </c>
+      <c r="L40" s="168">
+        <f t="shared" si="7"/>
+        <v>57</v>
+      </c>
+      <c r="M40" s="168">
+        <f t="shared" si="8"/>
+        <v>60</v>
+      </c>
+      <c r="N40" s="168">
+        <f t="shared" si="9"/>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="41" spans="2:16" x14ac:dyDescent="0.25">
       <c r="F41" s="169">
         <v>10</v>
       </c>
@@ -28542,8 +28790,46 @@
         <f t="shared" si="6"/>
         <v>214.625</v>
       </c>
-    </row>
-    <row r="43" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="J41" s="169">
+        <v>9</v>
+      </c>
+      <c r="K41" s="168">
+        <v>42</v>
+      </c>
+      <c r="L41" s="168">
+        <f t="shared" si="7"/>
+        <v>42</v>
+      </c>
+      <c r="M41" s="168">
+        <f t="shared" si="8"/>
+        <v>42</v>
+      </c>
+      <c r="N41" s="168">
+        <f t="shared" si="9"/>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="42" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="J42" s="169">
+        <v>10</v>
+      </c>
+      <c r="K42" s="168">
+        <v>74</v>
+      </c>
+      <c r="L42" s="168">
+        <f t="shared" si="7"/>
+        <v>72</v>
+      </c>
+      <c r="M42" s="168">
+        <f t="shared" si="8"/>
+        <v>75</v>
+      </c>
+      <c r="N42" s="168">
+        <f t="shared" si="9"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="43" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B43" s="260" t="s">
         <v>813</v>
       </c>
@@ -28555,7 +28841,7 @@
       <c r="G43" s="260"/>
       <c r="H43" s="260"/>
     </row>
-    <row r="44" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B44" s="167" t="s">
         <v>901</v>
       </c>
@@ -28575,7 +28861,7 @@
         <v>818</v>
       </c>
     </row>
-    <row r="45" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B45" s="169">
         <v>1</v>
       </c>
@@ -28595,8 +28881,17 @@
         <f t="array" ref="H45:H54">SMALL($G$45:$G$54,F45:F54)</f>
         <v>128</v>
       </c>
-    </row>
-    <row r="46" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="J45" s="260" t="s">
+        <v>913</v>
+      </c>
+      <c r="K45" s="260"/>
+      <c r="L45" s="260"/>
+      <c r="M45" s="260"/>
+      <c r="N45" s="260"/>
+      <c r="O45" s="260"/>
+      <c r="P45" s="260"/>
+    </row>
+    <row r="46" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B46" s="169">
         <v>2</v>
       </c>
@@ -28615,8 +28910,29 @@
       <c r="H46" s="168">
         <v>206</v>
       </c>
-    </row>
-    <row r="47" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="J46" s="167" t="s">
+        <v>901</v>
+      </c>
+      <c r="K46" s="167" t="s">
+        <v>902</v>
+      </c>
+      <c r="L46" s="267" t="s">
+        <v>914</v>
+      </c>
+      <c r="M46" s="167" t="s">
+        <v>878</v>
+      </c>
+      <c r="N46" s="265" t="s">
+        <v>883</v>
+      </c>
+      <c r="O46" s="265" t="s">
+        <v>888</v>
+      </c>
+      <c r="P46" s="265" t="s">
+        <v>893</v>
+      </c>
+    </row>
+    <row r="47" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B47" s="169">
         <v>3</v>
       </c>
@@ -28635,8 +28951,34 @@
       <c r="H47" s="168">
         <v>296</v>
       </c>
-    </row>
-    <row r="48" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="J47" s="169">
+        <v>1</v>
+      </c>
+      <c r="K47" s="168">
+        <v>49</v>
+      </c>
+      <c r="L47" s="168">
+        <f>-ABS(K47)</f>
+        <v>-49</v>
+      </c>
+      <c r="M47" s="168">
+        <f>ABS(L47)</f>
+        <v>49</v>
+      </c>
+      <c r="N47" s="168">
+        <f>MOD(K47,3)</f>
+        <v>1</v>
+      </c>
+      <c r="O47" s="168">
+        <f>POWER(J47,3)</f>
+        <v>1</v>
+      </c>
+      <c r="P47" s="168">
+        <f>ROUND(SQRT(K47),2)</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="48" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B48" s="169">
         <v>4</v>
       </c>
@@ -28655,8 +28997,34 @@
       <c r="H48" s="168">
         <v>330</v>
       </c>
-    </row>
-    <row r="49" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="J48" s="169">
+        <v>2</v>
+      </c>
+      <c r="K48" s="168">
+        <v>92</v>
+      </c>
+      <c r="L48" s="168">
+        <f t="shared" ref="L48:L56" si="10">-ABS(K48)</f>
+        <v>-92</v>
+      </c>
+      <c r="M48" s="168">
+        <f t="shared" ref="M48:M56" si="11">ABS(L48)</f>
+        <v>92</v>
+      </c>
+      <c r="N48" s="168">
+        <f t="shared" ref="N48:N56" si="12">MOD(K48,3)</f>
+        <v>2</v>
+      </c>
+      <c r="O48" s="168">
+        <f t="shared" ref="O48:O56" si="13">POWER(J48,3)</f>
+        <v>8</v>
+      </c>
+      <c r="P48" s="168">
+        <f t="shared" ref="P48:P56" si="14">SQRT(K48)</f>
+        <v>9.5916630466254382</v>
+      </c>
+    </row>
+    <row r="49" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B49" s="169">
         <v>5</v>
       </c>
@@ -28675,8 +29043,34 @@
       <c r="H49" s="168">
         <v>422</v>
       </c>
-    </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="J49" s="169">
+        <v>3</v>
+      </c>
+      <c r="K49" s="168">
+        <v>49</v>
+      </c>
+      <c r="L49" s="168">
+        <f t="shared" si="10"/>
+        <v>-49</v>
+      </c>
+      <c r="M49" s="168">
+        <f t="shared" si="11"/>
+        <v>49</v>
+      </c>
+      <c r="N49" s="168">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="O49" s="168">
+        <f t="shared" si="13"/>
+        <v>27</v>
+      </c>
+      <c r="P49" s="168">
+        <f t="shared" si="14"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="50" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B50" s="169">
         <v>6</v>
       </c>
@@ -28695,8 +29089,34 @@
       <c r="H50" s="168">
         <v>486</v>
       </c>
-    </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="J50" s="169">
+        <v>4</v>
+      </c>
+      <c r="K50" s="168">
+        <v>32</v>
+      </c>
+      <c r="L50" s="168">
+        <f t="shared" si="10"/>
+        <v>-32</v>
+      </c>
+      <c r="M50" s="168">
+        <f t="shared" si="11"/>
+        <v>32</v>
+      </c>
+      <c r="N50" s="168">
+        <f t="shared" si="12"/>
+        <v>2</v>
+      </c>
+      <c r="O50" s="168">
+        <f t="shared" si="13"/>
+        <v>64</v>
+      </c>
+      <c r="P50" s="168">
+        <f t="shared" si="14"/>
+        <v>5.6568542494923806</v>
+      </c>
+    </row>
+    <row r="51" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B51" s="169">
         <v>7</v>
       </c>
@@ -28715,8 +29135,34 @@
       <c r="H51" s="168">
         <v>528</v>
       </c>
-    </row>
-    <row r="52" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="J51" s="169">
+        <v>5</v>
+      </c>
+      <c r="K51" s="168">
+        <v>43</v>
+      </c>
+      <c r="L51" s="168">
+        <f t="shared" si="10"/>
+        <v>-43</v>
+      </c>
+      <c r="M51" s="168">
+        <f t="shared" si="11"/>
+        <v>43</v>
+      </c>
+      <c r="N51" s="168">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="O51" s="168">
+        <f t="shared" si="13"/>
+        <v>125</v>
+      </c>
+      <c r="P51" s="168">
+        <f t="shared" si="14"/>
+        <v>6.5574385243020004</v>
+      </c>
+    </row>
+    <row r="52" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B52" s="169">
         <v>8</v>
       </c>
@@ -28735,8 +29181,34 @@
       <c r="H52" s="168">
         <v>813</v>
       </c>
-    </row>
-    <row r="53" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="J52" s="169">
+        <v>6</v>
+      </c>
+      <c r="K52" s="168">
+        <v>57</v>
+      </c>
+      <c r="L52" s="168">
+        <f t="shared" si="10"/>
+        <v>-57</v>
+      </c>
+      <c r="M52" s="168">
+        <f t="shared" si="11"/>
+        <v>57</v>
+      </c>
+      <c r="N52" s="168">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="O52" s="168">
+        <f t="shared" si="13"/>
+        <v>216</v>
+      </c>
+      <c r="P52" s="168">
+        <f t="shared" si="14"/>
+        <v>7.5498344352707498</v>
+      </c>
+    </row>
+    <row r="53" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B53" s="169">
         <v>9</v>
       </c>
@@ -28755,8 +29227,34 @@
       <c r="H53" s="168">
         <v>821</v>
       </c>
-    </row>
-    <row r="54" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="J53" s="169">
+        <v>7</v>
+      </c>
+      <c r="K53" s="168">
+        <v>45</v>
+      </c>
+      <c r="L53" s="168">
+        <f t="shared" si="10"/>
+        <v>-45</v>
+      </c>
+      <c r="M53" s="168">
+        <f t="shared" si="11"/>
+        <v>45</v>
+      </c>
+      <c r="N53" s="168">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="O53" s="168">
+        <f t="shared" si="13"/>
+        <v>343</v>
+      </c>
+      <c r="P53" s="168">
+        <f>SQRT(K53)</f>
+        <v>6.7082039324993694</v>
+      </c>
+    </row>
+    <row r="54" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B54" s="169">
         <v>10</v>
       </c>
@@ -28775,13 +29273,97 @@
       <c r="H54" s="168">
         <v>942</v>
       </c>
+      <c r="J54" s="169">
+        <v>8</v>
+      </c>
+      <c r="K54" s="168">
+        <v>59</v>
+      </c>
+      <c r="L54" s="168">
+        <f t="shared" si="10"/>
+        <v>-59</v>
+      </c>
+      <c r="M54" s="168">
+        <f t="shared" si="11"/>
+        <v>59</v>
+      </c>
+      <c r="N54" s="168">
+        <f t="shared" si="12"/>
+        <v>2</v>
+      </c>
+      <c r="O54" s="168">
+        <f t="shared" si="13"/>
+        <v>512</v>
+      </c>
+      <c r="P54" s="168">
+        <f t="shared" si="14"/>
+        <v>7.6811457478686078</v>
+      </c>
+    </row>
+    <row r="55" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="J55" s="169">
+        <v>9</v>
+      </c>
+      <c r="K55" s="168">
+        <v>42</v>
+      </c>
+      <c r="L55" s="168">
+        <f t="shared" si="10"/>
+        <v>-42</v>
+      </c>
+      <c r="M55" s="168">
+        <f t="shared" si="11"/>
+        <v>42</v>
+      </c>
+      <c r="N55" s="168">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="O55" s="168">
+        <f t="shared" si="13"/>
+        <v>729</v>
+      </c>
+      <c r="P55" s="168">
+        <f t="shared" si="14"/>
+        <v>6.4807406984078604</v>
+      </c>
+    </row>
+    <row r="56" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="J56" s="169">
+        <v>10</v>
+      </c>
+      <c r="K56" s="168">
+        <v>74</v>
+      </c>
+      <c r="L56" s="168">
+        <f t="shared" si="10"/>
+        <v>-74</v>
+      </c>
+      <c r="M56" s="168">
+        <f t="shared" si="11"/>
+        <v>74</v>
+      </c>
+      <c r="N56" s="168">
+        <f t="shared" si="12"/>
+        <v>2</v>
+      </c>
+      <c r="O56" s="168">
+        <f t="shared" si="13"/>
+        <v>1000</v>
+      </c>
+      <c r="P56" s="168">
+        <f t="shared" si="14"/>
+        <v>8.6023252670426267</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="11">
+    <mergeCell ref="J45:P45"/>
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="B17:D17"/>
     <mergeCell ref="B30:D30"/>
     <mergeCell ref="B43:D43"/>
+    <mergeCell ref="J31:N31"/>
     <mergeCell ref="F43:H43"/>
     <mergeCell ref="F3:H3"/>
     <mergeCell ref="F17:H17"/>
@@ -28794,6 +29376,16 @@
   <conditionalFormatting sqref="G45:G54">
     <cfRule type="top10" dxfId="0" priority="2" bottom="1" rank="3"/>
   </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3797C5F0-736C-4467-B50E-FE7290689039}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -31252,11 +31844,11 @@
       </c>
       <c r="D2" s="25">
         <f t="shared" ref="C2:F15" ca="1" si="0">RANDBETWEEN(0,100)</f>
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E2" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>90</v>
+        <v>42</v>
       </c>
       <c r="F2" s="25"/>
       <c r="G2" s="28">
@@ -31278,16 +31870,16 @@
       </c>
       <c r="C3" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>96</v>
+        <v>57</v>
       </c>
       <c r="D3" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>65</v>
+        <v>24</v>
       </c>
       <c r="E3" s="25"/>
       <c r="F3" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="G3" s="28">
         <f t="shared" ref="G3:G15" ca="1" si="1">COUNT(C3:F3)</f>
@@ -31309,11 +31901,11 @@
       <c r="C4" s="25"/>
       <c r="D4" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>82</v>
+        <v>18</v>
       </c>
       <c r="E4" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>7</v>
+        <v>42</v>
       </c>
       <c r="F4" s="25"/>
       <c r="G4" s="28">
@@ -31335,16 +31927,16 @@
       </c>
       <c r="C5" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>1</v>
+        <v>89</v>
       </c>
       <c r="D5" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>93</v>
+        <v>39</v>
       </c>
       <c r="E5" s="25"/>
       <c r="F5" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>47</v>
+        <v>18</v>
       </c>
       <c r="G5" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -31365,16 +31957,16 @@
       </c>
       <c r="C6" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>8</v>
+        <v>95</v>
       </c>
       <c r="D6" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>6</v>
+        <v>98</v>
       </c>
       <c r="E6" s="25"/>
       <c r="F6" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="G6" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -31396,15 +31988,15 @@
       <c r="C7" s="25"/>
       <c r="D7" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="E7" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>27</v>
+        <v>64</v>
       </c>
       <c r="F7" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="G7" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -31425,7 +32017,7 @@
       </c>
       <c r="C8" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>13</v>
+        <v>71</v>
       </c>
       <c r="D8" s="25" t="s">
         <v>468</v>
@@ -31435,7 +32027,7 @@
       </c>
       <c r="F8" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="G8" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -31456,19 +32048,19 @@
       </c>
       <c r="C9" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="D9" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="E9" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>3</v>
+        <v>39</v>
       </c>
       <c r="F9" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>70</v>
+        <v>23</v>
       </c>
       <c r="G9" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -31489,12 +32081,12 @@
       </c>
       <c r="C10" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="D10" s="25"/>
       <c r="E10" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>19</v>
+        <v>69</v>
       </c>
       <c r="F10" s="25"/>
       <c r="G10" s="28">
@@ -31516,19 +32108,19 @@
       </c>
       <c r="C11" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="D11" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="E11" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="F11" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>76</v>
+        <v>56</v>
       </c>
       <c r="G11" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -31549,15 +32141,15 @@
       </c>
       <c r="C12" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="D12" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>52</v>
+        <v>84</v>
       </c>
       <c r="E12" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>99</v>
+        <v>53</v>
       </c>
       <c r="F12" s="25"/>
       <c r="G12" s="28">
@@ -31579,16 +32171,16 @@
       </c>
       <c r="C13" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D13" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="E13" s="25"/>
       <c r="F13" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G13" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -31609,18 +32201,18 @@
       </c>
       <c r="C14" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>5</v>
+        <v>90</v>
       </c>
       <c r="D14" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E14" s="25" t="s">
         <v>468</v>
       </c>
       <c r="F14" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="G14" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -31645,7 +32237,7 @@
       <c r="D15" s="27"/>
       <c r="E15" s="27">
         <f t="shared" ca="1" si="0"/>
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="F15" s="27" t="s">
         <v>468</v>
@@ -36082,54 +36674,54 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E51">
-    <cfRule type="cellIs" dxfId="59" priority="44" operator="equal">
+    <cfRule type="cellIs" dxfId="43" priority="44" operator="equal">
       <formula>20000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="58" priority="45" operator="between">
+    <cfRule type="cellIs" dxfId="42" priority="45" operator="between">
       <formula>50000</formula>
       <formula>100000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="57" priority="46" operator="between">
+    <cfRule type="cellIs" dxfId="41" priority="46" operator="between">
       <formula>"Rs. 65,984"</formula>
       <formula>"Rs. 121,395"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="56" priority="47" operator="lessThan">
+    <cfRule type="cellIs" dxfId="40" priority="47" operator="lessThan">
       <formula>93689</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="55" priority="48" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="39" priority="48" operator="greaterThan">
       <formula>93689</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="54" priority="49" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="38" priority="49" operator="greaterThan">
       <formula>"Rs. 93,689"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:B53">
-    <cfRule type="containsText" dxfId="53" priority="43" operator="containsText" text="Ayesha khan">
+    <cfRule type="containsText" dxfId="37" priority="43" operator="containsText" text="Ayesha khan">
       <formula>NOT(ISERROR(SEARCH("Ayesha khan",B2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:A53">
-    <cfRule type="timePeriod" dxfId="52" priority="41" timePeriod="yesterday">
+    <cfRule type="timePeriod" dxfId="36" priority="41" timePeriod="yesterday">
       <formula>FLOOR(A3,1)=TODAY()-1</formula>
     </cfRule>
-    <cfRule type="timePeriod" dxfId="51" priority="42" timePeriod="yesterday">
+    <cfRule type="timePeriod" dxfId="35" priority="42" timePeriod="yesterday">
       <formula>FLOOR(A3,1)=TODAY()-1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:A53">
-    <cfRule type="timePeriod" dxfId="50" priority="38" timePeriod="nextWeek">
+    <cfRule type="timePeriod" dxfId="34" priority="38" timePeriod="nextWeek">
       <formula>AND(ROUNDDOWN(A2,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(A2,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
     </cfRule>
-    <cfRule type="timePeriod" dxfId="49" priority="39" timePeriod="yesterday">
+    <cfRule type="timePeriod" dxfId="33" priority="39" timePeriod="yesterday">
       <formula>FLOOR(A2,1)=TODAY()-1</formula>
     </cfRule>
-    <cfRule type="timePeriod" dxfId="48" priority="40" timePeriod="today">
+    <cfRule type="timePeriod" dxfId="32" priority="40" timePeriod="today">
       <formula>FLOOR(A2,1)=TODAY()</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F53">
-    <cfRule type="uniqueValues" dxfId="47" priority="36"/>
-    <cfRule type="duplicateValues" dxfId="46" priority="37"/>
+    <cfRule type="uniqueValues" dxfId="31" priority="36"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="37"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E55:E105">
     <cfRule type="dataBar" priority="18">

</xml_diff>